<commit_message>
Add Concentradora SSO integration and sync engineering project files
</commit_message>
<xml_diff>
--- a/src/Proyectos/11-B-9016-01/Rev_R0/FactorK_30/Espesor_0.105/11-B-9016-01-(12gacr ANSI-61) - K30 - V0-R0.xlsx
+++ b/src/Proyectos/11-B-9016-01/Rev_R0/FactorK_30/Espesor_0.105/11-B-9016-01-(12gacr ANSI-61) - K30 - V0-R0.xlsx
@@ -152,16 +152,6 @@
 
 <file path=xl/revisions/revisionHeaders.xml><?xml version="1.0" encoding="utf-8"?>
 <headers xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac" guid="{508E8EBD-2A39-4366-B470-C8FACCA0D270}" diskRevisions="1" revisionId="92" version="5">
-  <header guid="{EC8B92E7-782F-4B67-8193-8ABBE7F506A8}" dateTime="2026-06-05T11:43:28" maxSheetId="2" userName="Estacion Maquinados" r:id="rId1">
-    <sheetIdMap count="1">
-      <sheetId val="1"/>
-    </sheetIdMap>
-  </header>
-  <header guid="{7B93181E-5047-4D0C-9820-A1F71F841844}" dateTime="2026-06-05T12:43:54" maxSheetId="2" userName="Estacion Maquinados" r:id="rId2" minRId="1" maxRId="24">
-    <sheetIdMap count="1">
-      <sheetId val="1"/>
-    </sheetIdMap>
-  </header>
   <header guid="{AD579068-09A7-4F33-B88F-213BC84A7D0A}" dateTime="2026-06-19T16:34:34" maxSheetId="3" userName="Estacion Maquinados" r:id="rId3" minRId="25" maxRId="55">
     <sheetIdMap count="2">
       <sheetId val="1"/>
@@ -181,594 +171,6 @@
     </sheetIdMap>
   </header>
 </headers>
-</file>
-
-<file path=xl/revisions/revisionLog1.xml><?xml version="1.0" encoding="utf-8"?>
-<revisions xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac"/>
-</file>
-
-<file path=xl/revisions/revisionLog2.xml><?xml version="1.0" encoding="utf-8"?>
-<revisions xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <rfmt sheetId="1" sqref="B2:B10">
-    <dxf>
-      <numFmt numFmtId="166" formatCode="0.000"/>
-    </dxf>
-  </rfmt>
-  <rcc rId="1" sId="1" odxf="1" dxf="1">
-    <oc r="C2">
-      <v>1.2849999999999999</v>
-    </oc>
-    <nc r="C2">
-      <f>B2-0.015</f>
-    </nc>
-    <ndxf>
-      <numFmt numFmtId="166" formatCode="0.000"/>
-    </ndxf>
-  </rcc>
-  <rcc rId="2" sId="1" odxf="1" dxf="1">
-    <oc r="D2">
-      <v>1.3149999999999999</v>
-    </oc>
-    <nc r="D2">
-      <f>B2+0.015</f>
-    </nc>
-    <ndxf>
-      <numFmt numFmtId="166" formatCode="0.000"/>
-    </ndxf>
-  </rcc>
-  <rcc rId="3" sId="1" odxf="1" dxf="1">
-    <oc r="C3">
-      <v>1.2350000000000001</v>
-    </oc>
-    <nc r="C3">
-      <f>B3-0.015</f>
-    </nc>
-    <ndxf>
-      <numFmt numFmtId="166" formatCode="0.000"/>
-    </ndxf>
-  </rcc>
-  <rcc rId="4" sId="1" odxf="1" dxf="1">
-    <oc r="C4">
-      <v>2.2349999999999999</v>
-    </oc>
-    <nc r="C4">
-      <f>B4-0.015</f>
-    </nc>
-    <ndxf>
-      <numFmt numFmtId="166" formatCode="0.000"/>
-    </ndxf>
-  </rcc>
-  <rcc rId="5" sId="1" odxf="1" dxf="1">
-    <oc r="C5">
-      <v>0.26500000000000001</v>
-    </oc>
-    <nc r="C5">
-      <f>B5-0.015</f>
-    </nc>
-    <ndxf>
-      <numFmt numFmtId="166" formatCode="0.000"/>
-    </ndxf>
-  </rcc>
-  <rcc rId="6" sId="1" odxf="1" dxf="1">
-    <oc r="C6">
-      <v>1.675</v>
-    </oc>
-    <nc r="C6">
-      <f>B6-0.015</f>
-    </nc>
-    <ndxf>
-      <numFmt numFmtId="166" formatCode="0.000"/>
-    </ndxf>
-  </rcc>
-  <rcc rId="7" sId="1" odxf="1" dxf="1">
-    <oc r="C7">
-      <v>0.73499999999999999</v>
-    </oc>
-    <nc r="C7">
-      <f>B7-0.015</f>
-    </nc>
-    <ndxf>
-      <numFmt numFmtId="166" formatCode="0.000"/>
-    </ndxf>
-  </rcc>
-  <rcc rId="8" sId="1" odxf="1" dxf="1">
-    <oc r="C8">
-      <v>0.79500000000000004</v>
-    </oc>
-    <nc r="C8">
-      <f>B8-0.015</f>
-    </nc>
-    <ndxf>
-      <numFmt numFmtId="166" formatCode="0.000"/>
-    </ndxf>
-  </rcc>
-  <rcc rId="9" sId="1" odxf="1" dxf="1">
-    <oc r="C9">
-      <v>0.36499999999999999</v>
-    </oc>
-    <nc r="C9">
-      <f>B9-0.015</f>
-    </nc>
-    <ndxf>
-      <numFmt numFmtId="166" formatCode="0.000"/>
-    </ndxf>
-  </rcc>
-  <rcc rId="10" sId="1" odxf="1" dxf="1">
-    <oc r="C10">
-      <v>0.19500000000000001</v>
-    </oc>
-    <nc r="C10">
-      <f>B10-0.015</f>
-    </nc>
-    <ndxf>
-      <numFmt numFmtId="166" formatCode="0.000"/>
-    </ndxf>
-  </rcc>
-  <rcc rId="11" sId="1" odxf="1" dxf="1">
-    <oc r="D3">
-      <v>1.2649999999999999</v>
-    </oc>
-    <nc r="D3">
-      <f>B3+0.015</f>
-    </nc>
-    <ndxf>
-      <numFmt numFmtId="166" formatCode="0.000"/>
-    </ndxf>
-  </rcc>
-  <rcc rId="12" sId="1" odxf="1" dxf="1">
-    <oc r="D4">
-      <v>2.2650000000000001</v>
-    </oc>
-    <nc r="D4">
-      <f>B4+0.015</f>
-    </nc>
-    <ndxf>
-      <numFmt numFmtId="166" formatCode="0.000"/>
-    </ndxf>
-  </rcc>
-  <rcc rId="13" sId="1" odxf="1" dxf="1">
-    <oc r="D5">
-      <v>0.29499999999999998</v>
-    </oc>
-    <nc r="D5">
-      <f>B5+0.015</f>
-    </nc>
-    <ndxf>
-      <numFmt numFmtId="166" formatCode="0.000"/>
-    </ndxf>
-  </rcc>
-  <rcc rId="14" sId="1" odxf="1" dxf="1">
-    <oc r="D6">
-      <v>1.7050000000000001</v>
-    </oc>
-    <nc r="D6">
-      <f>B6+0.015</f>
-    </nc>
-    <ndxf>
-      <numFmt numFmtId="166" formatCode="0.000"/>
-    </ndxf>
-  </rcc>
-  <rcc rId="15" sId="1" odxf="1" dxf="1">
-    <oc r="D7">
-      <v>0.76500000000000001</v>
-    </oc>
-    <nc r="D7">
-      <f>B7+0.015</f>
-    </nc>
-    <ndxf>
-      <numFmt numFmtId="166" formatCode="0.000"/>
-    </ndxf>
-  </rcc>
-  <rcc rId="16" sId="1" odxf="1" dxf="1">
-    <oc r="D8">
-      <v>0.82499999999999996</v>
-    </oc>
-    <nc r="D8">
-      <f>B8+0.015</f>
-    </nc>
-    <ndxf>
-      <numFmt numFmtId="166" formatCode="0.000"/>
-    </ndxf>
-  </rcc>
-  <rcc rId="17" sId="1" odxf="1" dxf="1">
-    <oc r="D9">
-      <v>0.39500000000000002</v>
-    </oc>
-    <nc r="D9">
-      <f>B9+0.015</f>
-    </nc>
-    <ndxf>
-      <numFmt numFmtId="166" formatCode="0.000"/>
-    </ndxf>
-  </rcc>
-  <rcc rId="18" sId="1" odxf="1" dxf="1">
-    <oc r="D10">
-      <v>0.22500000000000001</v>
-    </oc>
-    <nc r="D10">
-      <f>B10+0.015</f>
-    </nc>
-    <ndxf>
-      <numFmt numFmtId="166" formatCode="0.000"/>
-    </ndxf>
-  </rcc>
-  <rfmt sheetId="1" sqref="A1:H10" start="0" length="2147483647">
-    <dxf>
-      <font>
-        <sz val="12"/>
-      </font>
-    </dxf>
-  </rfmt>
-  <rfmt sheetId="1" sqref="A1:H10" start="0" length="2147483647">
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
-    </dxf>
-  </rfmt>
-  <rfmt sheetId="1" sqref="A1:A10" start="0" length="0">
-    <dxf>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-      </border>
-    </dxf>
-  </rfmt>
-  <rfmt sheetId="1" sqref="A1:H1" start="0" length="0">
-    <dxf>
-      <border>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-  </rfmt>
-  <rfmt sheetId="1" sqref="H1:H10" start="0" length="0">
-    <dxf>
-      <border>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-      </border>
-    </dxf>
-  </rfmt>
-  <rfmt sheetId="1" sqref="A10:H10" start="0" length="0">
-    <dxf>
-      <border>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-  </rfmt>
-  <rfmt sheetId="1" sqref="A1:H10">
-    <dxf>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-  </rfmt>
-  <rcc rId="19" sId="1" numFmtId="4">
-    <oc r="B9">
-      <v>0.38</v>
-    </oc>
-    <nc r="B9">
-      <v>0.92200000000000004</v>
-    </nc>
-  </rcc>
-  <rrc rId="20" sId="1" eol="1" ref="A11:XFD11" action="insertRow"/>
-  <rfmt sheetId="1" sqref="A11">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-  </rfmt>
-  <rfmt sheetId="1" sqref="B11">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="166" formatCode="0.000"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-  </rfmt>
-  <rfmt sheetId="1" sqref="C11">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="166" formatCode="0.000"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-  </rfmt>
-  <rfmt sheetId="1" sqref="D11">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="166" formatCode="0.000"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-  </rfmt>
-  <rcc rId="21" sId="1" odxf="1" dxf="1">
-    <nc r="A11" t="inlineStr">
-      <is>
-        <t>J</t>
-      </is>
-    </nc>
-    <ndxf>
-      <border outline="0">
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </ndxf>
-  </rcc>
-  <rcc rId="22" sId="1" odxf="1" dxf="1" numFmtId="4">
-    <nc r="B11">
-      <v>0.81</v>
-    </nc>
-    <ndxf>
-      <border outline="0">
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </ndxf>
-  </rcc>
-  <rcc rId="23" sId="1" odxf="1" dxf="1">
-    <nc r="C11">
-      <f>B11-0.015</f>
-    </nc>
-    <ndxf>
-      <border outline="0">
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </ndxf>
-  </rcc>
-  <rcc rId="24" sId="1" odxf="1" dxf="1">
-    <nc r="D11">
-      <f>B11+0.015</f>
-    </nc>
-    <ndxf>
-      <border outline="0">
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </ndxf>
-  </rcc>
-  <rfmt sheetId="1" sqref="E11" start="0" length="0">
-    <dxf>
-      <font>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-  </rfmt>
-  <rfmt sheetId="1" sqref="F11" start="0" length="0">
-    <dxf>
-      <font>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-  </rfmt>
-  <rfmt sheetId="1" sqref="G11" start="0" length="0">
-    <dxf>
-      <font>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-  </rfmt>
-  <rfmt sheetId="1" sqref="H11" start="0" length="0">
-    <dxf>
-      <font>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Century Gothic"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <border outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-  </rfmt>
-</revisions>
 </file>
 
 <file path=xl/revisions/revisionLog3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>